<commit_message>
Adding reading abordados base prata and ouro
</commit_message>
<xml_diff>
--- a/arquivos/bb_municipio_estacao.xlsx
+++ b/arquivos/bb_municipio_estacao.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\F257064\Documents\Codes\NEW_NFV\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\F257064\Documents\Codes\atualizacao nfv automatico\NEW_NFV\arquivos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{214B09D6-D1F6-45D2-AD1D-50D972E2CB32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F450C2F-1680-44C0-B311-C444D6062868}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-24120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -690,9 +690,6 @@
     <t>TTE SC</t>
   </si>
   <si>
-    <t>TSA NA</t>
-  </si>
-  <si>
     <t>URA FR</t>
   </si>
   <si>
@@ -718,6 +715,9 @@
   </si>
   <si>
     <t>ESTACAO</t>
+  </si>
+  <si>
+    <t>TSA AN</t>
   </si>
 </sst>
 </file>
@@ -753,9 +753,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1044,13 +1043,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>227</v>
+      </c>
+      <c r="B1" t="s">
         <v>228</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>229</v>
-      </c>
-      <c r="C1" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -1548,14 +1547,14 @@
         <v>146</v>
       </c>
     </row>
-    <row r="47" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="B47" t="s">
         <v>34</v>
       </c>
-      <c r="C47" s="1" t="s">
+      <c r="C47" t="s">
         <v>147</v>
       </c>
     </row>
@@ -1566,7 +1565,7 @@
       <c r="B48" t="s">
         <v>35</v>
       </c>
-      <c r="C48" s="1" t="s">
+      <c r="C48" t="s">
         <v>148</v>
       </c>
     </row>
@@ -1577,7 +1576,7 @@
       <c r="B49" t="s">
         <v>36</v>
       </c>
-      <c r="C49" s="1" t="s">
+      <c r="C49" t="s">
         <v>149</v>
       </c>
     </row>
@@ -1588,7 +1587,7 @@
       <c r="B50" t="s">
         <v>36</v>
       </c>
-      <c r="C50" s="1" t="s">
+      <c r="C50" t="s">
         <v>150</v>
       </c>
     </row>
@@ -1599,7 +1598,7 @@
       <c r="B51" t="s">
         <v>37</v>
       </c>
-      <c r="C51" s="1" t="s">
+      <c r="C51" t="s">
         <v>151</v>
       </c>
     </row>
@@ -1610,7 +1609,7 @@
       <c r="B52" t="s">
         <v>37</v>
       </c>
-      <c r="C52" s="1" t="s">
+      <c r="C52" t="s">
         <v>152</v>
       </c>
     </row>
@@ -1621,7 +1620,7 @@
       <c r="B53" t="s">
         <v>38</v>
       </c>
-      <c r="C53" s="1" t="s">
+      <c r="C53" t="s">
         <v>153</v>
       </c>
     </row>
@@ -1632,7 +1631,7 @@
       <c r="B54" t="s">
         <v>39</v>
       </c>
-      <c r="C54" s="1" t="s">
+      <c r="C54" t="s">
         <v>154</v>
       </c>
     </row>
@@ -1643,7 +1642,7 @@
       <c r="B55" t="s">
         <v>40</v>
       </c>
-      <c r="C55" s="1" t="s">
+      <c r="C55" t="s">
         <v>155</v>
       </c>
     </row>
@@ -1654,7 +1653,7 @@
       <c r="B56" t="s">
         <v>41</v>
       </c>
-      <c r="C56" s="1" t="s">
+      <c r="C56" t="s">
         <v>156</v>
       </c>
     </row>
@@ -1665,7 +1664,7 @@
       <c r="B57" t="s">
         <v>42</v>
       </c>
-      <c r="C57" s="1" t="s">
+      <c r="C57" t="s">
         <v>157</v>
       </c>
     </row>
@@ -1676,7 +1675,7 @@
       <c r="B58" t="s">
         <v>43</v>
       </c>
-      <c r="C58" s="1" t="s">
+      <c r="C58" t="s">
         <v>158</v>
       </c>
     </row>
@@ -1687,7 +1686,7 @@
       <c r="B59" t="s">
         <v>44</v>
       </c>
-      <c r="C59" s="1" t="s">
+      <c r="C59" t="s">
         <v>159</v>
       </c>
     </row>
@@ -1698,7 +1697,7 @@
       <c r="B60" t="s">
         <v>45</v>
       </c>
-      <c r="C60" s="1" t="s">
+      <c r="C60" t="s">
         <v>160</v>
       </c>
     </row>
@@ -1709,7 +1708,7 @@
       <c r="B61" t="s">
         <v>46</v>
       </c>
-      <c r="C61" s="1" t="s">
+      <c r="C61" t="s">
         <v>161</v>
       </c>
     </row>
@@ -1720,7 +1719,7 @@
       <c r="B62" t="s">
         <v>47</v>
       </c>
-      <c r="C62" s="1" t="s">
+      <c r="C62" t="s">
         <v>162</v>
       </c>
     </row>
@@ -1731,7 +1730,7 @@
       <c r="B63" t="s">
         <v>48</v>
       </c>
-      <c r="C63" s="1" t="s">
+      <c r="C63" t="s">
         <v>163</v>
       </c>
     </row>
@@ -1742,7 +1741,7 @@
       <c r="B64" t="s">
         <v>49</v>
       </c>
-      <c r="C64" s="1" t="s">
+      <c r="C64" t="s">
         <v>164</v>
       </c>
     </row>
@@ -1753,7 +1752,7 @@
       <c r="B65" t="s">
         <v>50</v>
       </c>
-      <c r="C65" s="1" t="s">
+      <c r="C65" t="s">
         <v>165</v>
       </c>
     </row>
@@ -1764,7 +1763,7 @@
       <c r="B66" t="s">
         <v>51</v>
       </c>
-      <c r="C66" s="1" t="s">
+      <c r="C66" t="s">
         <v>166</v>
       </c>
     </row>
@@ -1775,7 +1774,7 @@
       <c r="B67" t="s">
         <v>52</v>
       </c>
-      <c r="C67" s="1" t="s">
+      <c r="C67" t="s">
         <v>167</v>
       </c>
     </row>
@@ -1786,7 +1785,7 @@
       <c r="B68" t="s">
         <v>53</v>
       </c>
-      <c r="C68" s="1" t="s">
+      <c r="C68" t="s">
         <v>168</v>
       </c>
     </row>
@@ -1797,7 +1796,7 @@
       <c r="B69" t="s">
         <v>53</v>
       </c>
-      <c r="C69" s="1" t="s">
+      <c r="C69" t="s">
         <v>169</v>
       </c>
     </row>
@@ -1808,7 +1807,7 @@
       <c r="B70" t="s">
         <v>54</v>
       </c>
-      <c r="C70" s="1" t="s">
+      <c r="C70" t="s">
         <v>170</v>
       </c>
     </row>
@@ -1819,7 +1818,7 @@
       <c r="B71" t="s">
         <v>54</v>
       </c>
-      <c r="C71" s="1" t="s">
+      <c r="C71" t="s">
         <v>171</v>
       </c>
     </row>
@@ -1830,7 +1829,7 @@
       <c r="B72" t="s">
         <v>54</v>
       </c>
-      <c r="C72" s="1" t="s">
+      <c r="C72" t="s">
         <v>172</v>
       </c>
     </row>
@@ -1841,7 +1840,7 @@
       <c r="B73" t="s">
         <v>55</v>
       </c>
-      <c r="C73" s="1" t="s">
+      <c r="C73" t="s">
         <v>173</v>
       </c>
     </row>
@@ -1852,7 +1851,7 @@
       <c r="B74" t="s">
         <v>56</v>
       </c>
-      <c r="C74" s="1" t="s">
+      <c r="C74" t="s">
         <v>174</v>
       </c>
     </row>
@@ -1863,7 +1862,7 @@
       <c r="B75" t="s">
         <v>57</v>
       </c>
-      <c r="C75" s="1" t="s">
+      <c r="C75" t="s">
         <v>175</v>
       </c>
     </row>
@@ -1874,7 +1873,7 @@
       <c r="B76" t="s">
         <v>58</v>
       </c>
-      <c r="C76" s="1" t="s">
+      <c r="C76" t="s">
         <v>176</v>
       </c>
     </row>
@@ -1885,7 +1884,7 @@
       <c r="B77" t="s">
         <v>59</v>
       </c>
-      <c r="C77" s="1" t="s">
+      <c r="C77" t="s">
         <v>177</v>
       </c>
     </row>
@@ -1896,7 +1895,7 @@
       <c r="B78" t="s">
         <v>60</v>
       </c>
-      <c r="C78" s="1" t="s">
+      <c r="C78" t="s">
         <v>178</v>
       </c>
     </row>
@@ -1907,7 +1906,7 @@
       <c r="B79" t="s">
         <v>61</v>
       </c>
-      <c r="C79" s="1" t="s">
+      <c r="C79" t="s">
         <v>179</v>
       </c>
     </row>
@@ -1918,7 +1917,7 @@
       <c r="B80" t="s">
         <v>62</v>
       </c>
-      <c r="C80" s="1" t="s">
+      <c r="C80" t="s">
         <v>180</v>
       </c>
     </row>
@@ -1929,7 +1928,7 @@
       <c r="B81" t="s">
         <v>63</v>
       </c>
-      <c r="C81" s="1" t="s">
+      <c r="C81" t="s">
         <v>181</v>
       </c>
     </row>
@@ -1940,7 +1939,7 @@
       <c r="B82" t="s">
         <v>64</v>
       </c>
-      <c r="C82" s="1" t="s">
+      <c r="C82" t="s">
         <v>182</v>
       </c>
     </row>
@@ -1951,7 +1950,7 @@
       <c r="B83" t="s">
         <v>65</v>
       </c>
-      <c r="C83" s="1" t="s">
+      <c r="C83" t="s">
         <v>183</v>
       </c>
     </row>
@@ -1962,7 +1961,7 @@
       <c r="B84" t="s">
         <v>66</v>
       </c>
-      <c r="C84" s="1" t="s">
+      <c r="C84" t="s">
         <v>184</v>
       </c>
     </row>
@@ -1973,7 +1972,7 @@
       <c r="B85" t="s">
         <v>67</v>
       </c>
-      <c r="C85" s="1" t="s">
+      <c r="C85" t="s">
         <v>185</v>
       </c>
     </row>
@@ -1984,7 +1983,7 @@
       <c r="B86" t="s">
         <v>68</v>
       </c>
-      <c r="C86" s="1" t="s">
+      <c r="C86" t="s">
         <v>186</v>
       </c>
     </row>
@@ -1995,7 +1994,7 @@
       <c r="B87" t="s">
         <v>69</v>
       </c>
-      <c r="C87" s="1" t="s">
+      <c r="C87" t="s">
         <v>187</v>
       </c>
     </row>
@@ -2006,7 +2005,7 @@
       <c r="B88" t="s">
         <v>70</v>
       </c>
-      <c r="C88" s="1" t="s">
+      <c r="C88" t="s">
         <v>188</v>
       </c>
     </row>
@@ -2017,7 +2016,7 @@
       <c r="B89" t="s">
         <v>71</v>
       </c>
-      <c r="C89" s="1" t="s">
+      <c r="C89" t="s">
         <v>189</v>
       </c>
     </row>
@@ -2028,7 +2027,7 @@
       <c r="B90" t="s">
         <v>71</v>
       </c>
-      <c r="C90" s="1" t="s">
+      <c r="C90" t="s">
         <v>190</v>
       </c>
     </row>
@@ -2039,7 +2038,7 @@
       <c r="B91" t="s">
         <v>72</v>
       </c>
-      <c r="C91" s="1" t="s">
+      <c r="C91" t="s">
         <v>191</v>
       </c>
     </row>
@@ -2050,7 +2049,7 @@
       <c r="B92" t="s">
         <v>73</v>
       </c>
-      <c r="C92" s="1" t="s">
+      <c r="C92" t="s">
         <v>192</v>
       </c>
     </row>
@@ -2061,7 +2060,7 @@
       <c r="B93" t="s">
         <v>73</v>
       </c>
-      <c r="C93" s="1" t="s">
+      <c r="C93" t="s">
         <v>193</v>
       </c>
     </row>
@@ -2072,7 +2071,7 @@
       <c r="B94" t="s">
         <v>74</v>
       </c>
-      <c r="C94" s="1" t="s">
+      <c r="C94" t="s">
         <v>194</v>
       </c>
     </row>
@@ -2083,7 +2082,7 @@
       <c r="B95" t="s">
         <v>75</v>
       </c>
-      <c r="C95" s="1" t="s">
+      <c r="C95" t="s">
         <v>195</v>
       </c>
     </row>
@@ -2094,7 +2093,7 @@
       <c r="B96" t="s">
         <v>75</v>
       </c>
-      <c r="C96" s="1" t="s">
+      <c r="C96" t="s">
         <v>196</v>
       </c>
     </row>
@@ -2105,7 +2104,7 @@
       <c r="B97" t="s">
         <v>76</v>
       </c>
-      <c r="C97" s="1" t="s">
+      <c r="C97" t="s">
         <v>197</v>
       </c>
     </row>
@@ -2116,7 +2115,7 @@
       <c r="B98" t="s">
         <v>77</v>
       </c>
-      <c r="C98" s="1" t="s">
+      <c r="C98" t="s">
         <v>198</v>
       </c>
     </row>
@@ -2127,7 +2126,7 @@
       <c r="B99" t="s">
         <v>77</v>
       </c>
-      <c r="C99" s="1" t="s">
+      <c r="C99" t="s">
         <v>199</v>
       </c>
     </row>
@@ -2138,7 +2137,7 @@
       <c r="B100" t="s">
         <v>77</v>
       </c>
-      <c r="C100" s="1" t="s">
+      <c r="C100" t="s">
         <v>200</v>
       </c>
     </row>
@@ -2149,7 +2148,7 @@
       <c r="B101" t="s">
         <v>78</v>
       </c>
-      <c r="C101" s="1" t="s">
+      <c r="C101" t="s">
         <v>201</v>
       </c>
     </row>
@@ -2160,7 +2159,7 @@
       <c r="B102" t="s">
         <v>79</v>
       </c>
-      <c r="C102" s="1" t="s">
+      <c r="C102" t="s">
         <v>202</v>
       </c>
     </row>
@@ -2171,7 +2170,7 @@
       <c r="B103" t="s">
         <v>80</v>
       </c>
-      <c r="C103" s="1" t="s">
+      <c r="C103" t="s">
         <v>203</v>
       </c>
     </row>
@@ -2182,7 +2181,7 @@
       <c r="B104" t="s">
         <v>81</v>
       </c>
-      <c r="C104" s="1" t="s">
+      <c r="C104" t="s">
         <v>204</v>
       </c>
     </row>
@@ -2193,7 +2192,7 @@
       <c r="B105" t="s">
         <v>82</v>
       </c>
-      <c r="C105" s="1" t="s">
+      <c r="C105" t="s">
         <v>205</v>
       </c>
     </row>
@@ -2204,7 +2203,7 @@
       <c r="B106" t="s">
         <v>83</v>
       </c>
-      <c r="C106" s="1" t="s">
+      <c r="C106" t="s">
         <v>206</v>
       </c>
     </row>
@@ -2215,7 +2214,7 @@
       <c r="B107" t="s">
         <v>84</v>
       </c>
-      <c r="C107" s="1" t="s">
+      <c r="C107" t="s">
         <v>207</v>
       </c>
     </row>
@@ -2226,7 +2225,7 @@
       <c r="B108" t="s">
         <v>85</v>
       </c>
-      <c r="C108" s="1" t="s">
+      <c r="C108" t="s">
         <v>208</v>
       </c>
     </row>
@@ -2237,7 +2236,7 @@
       <c r="B109" t="s">
         <v>86</v>
       </c>
-      <c r="C109" s="1" t="s">
+      <c r="C109" t="s">
         <v>209</v>
       </c>
     </row>
@@ -2248,7 +2247,7 @@
       <c r="B110" t="s">
         <v>87</v>
       </c>
-      <c r="C110" s="1" t="s">
+      <c r="C110" t="s">
         <v>210</v>
       </c>
     </row>
@@ -2259,7 +2258,7 @@
       <c r="B111" t="s">
         <v>88</v>
       </c>
-      <c r="C111" s="1" t="s">
+      <c r="C111" t="s">
         <v>211</v>
       </c>
     </row>
@@ -2270,7 +2269,7 @@
       <c r="B112" t="s">
         <v>89</v>
       </c>
-      <c r="C112" s="1" t="s">
+      <c r="C112" t="s">
         <v>212</v>
       </c>
     </row>
@@ -2281,7 +2280,7 @@
       <c r="B113" t="s">
         <v>90</v>
       </c>
-      <c r="C113" s="1" t="s">
+      <c r="C113" t="s">
         <v>213</v>
       </c>
     </row>
@@ -2292,7 +2291,7 @@
       <c r="B114" t="s">
         <v>91</v>
       </c>
-      <c r="C114" s="1" t="s">
+      <c r="C114" t="s">
         <v>214</v>
       </c>
     </row>
@@ -2303,7 +2302,7 @@
       <c r="B115" t="s">
         <v>91</v>
       </c>
-      <c r="C115" s="1" t="s">
+      <c r="C115" t="s">
         <v>215</v>
       </c>
     </row>
@@ -2314,7 +2313,7 @@
       <c r="B116" t="s">
         <v>91</v>
       </c>
-      <c r="C116" s="1" t="s">
+      <c r="C116" t="s">
         <v>216</v>
       </c>
     </row>
@@ -2325,7 +2324,7 @@
       <c r="B117" t="s">
         <v>91</v>
       </c>
-      <c r="C117" s="1" t="s">
+      <c r="C117" t="s">
         <v>217</v>
       </c>
     </row>
@@ -2336,7 +2335,7 @@
       <c r="B118" t="s">
         <v>92</v>
       </c>
-      <c r="C118" s="1" t="s">
+      <c r="C118" t="s">
         <v>218</v>
       </c>
     </row>
@@ -2347,7 +2346,7 @@
       <c r="B119" t="s">
         <v>93</v>
       </c>
-      <c r="C119" s="1" t="s">
+      <c r="C119" t="s">
         <v>219</v>
       </c>
     </row>
@@ -2358,7 +2357,7 @@
       <c r="B120" t="s">
         <v>94</v>
       </c>
-      <c r="C120" s="1" t="s">
+      <c r="C120" t="s">
         <v>220</v>
       </c>
     </row>
@@ -2369,8 +2368,8 @@
       <c r="B121" t="s">
         <v>95</v>
       </c>
-      <c r="C121" s="1" t="s">
-        <v>221</v>
+      <c r="C121" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.3">
@@ -2380,8 +2379,8 @@
       <c r="B122" t="s">
         <v>96</v>
       </c>
-      <c r="C122" s="1" t="s">
-        <v>222</v>
+      <c r="C122" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.3">
@@ -2391,8 +2390,8 @@
       <c r="B123" t="s">
         <v>97</v>
       </c>
-      <c r="C123" s="1" t="s">
-        <v>223</v>
+      <c r="C123" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.3">
@@ -2402,8 +2401,8 @@
       <c r="B124" t="s">
         <v>98</v>
       </c>
-      <c r="C124" s="1" t="s">
-        <v>224</v>
+      <c r="C124" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.3">
@@ -2413,8 +2412,8 @@
       <c r="B125" t="s">
         <v>99</v>
       </c>
-      <c r="C125" s="1" t="s">
-        <v>225</v>
+      <c r="C125" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.3">
@@ -2424,8 +2423,8 @@
       <c r="B126" t="s">
         <v>100</v>
       </c>
-      <c r="C126" s="1" t="s">
-        <v>226</v>
+      <c r="C126" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.3">
@@ -2435,8 +2434,8 @@
       <c r="B127" t="s">
         <v>101</v>
       </c>
-      <c r="C127" s="1" t="s">
-        <v>227</v>
+      <c r="C127" t="s">
+        <v>226</v>
       </c>
     </row>
   </sheetData>

</xml_diff>